<commit_message>
Add Popular Cars USA & Canada Top 50 pipeline and complete first 3 videos (Ford F-150, Silverado, RAV4) with logo and sound (no outro)
</commit_message>
<xml_diff>
--- a/master_vehicles_tracker.xlsx
+++ b/master_vehicles_tracker.xlsx
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Real-time status across Generation, Editing, and Uploading | Last updated: 2026-09-21 00:30:23</t>
+          <t>Real-time status across Generation, Editing, and Uploading | Last updated: 2026-09-23 18:06:22</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="J10" s="11" t="inlineStr">
         <is>
-          <t>output\100_popular_cars_in_India_03_Maruti_Suzuki_Wagon_R\Maruti_Suzuki_Wagon_R.mp4</t>
+          <t>output\Popular_Cars_USA_Canada_Top_50_03_Toyota_RAV4\Toyota_RAV4.mp4</t>
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr">

</xml_diff>